<commit_message>
Add 11 source-reviewed NJU profiles with preserved retirement and guidance scope
</commit_message>
<xml_diff>
--- a/site/exports/nju-math.xlsx
+++ b/site/exports/nju-math.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -451,7 +451,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="57.4" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
     <col width="37.8" customWidth="1" min="7" max="7"/>
     <col width="26.6" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
@@ -569,10 +569,64 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>数学系</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>个人页原教授、博导及Department of Mathematics, Nanjing University／数学系明确职业身份；导航按同校数学学科复用数学学院节点，不认证数学系与学院法律同一、行政关系或更名，原数学系标签不被覆盖；博导是指导他人资格，不是本人导师。独立目录、现职未核实。；博士学习终2011-06与北京大学博士后始2011-04重叠，保留原区间，不推提前毕业或授位月份。；原空任职数组只表示未结构化其他职业经历，不表示没有工作；原简介职业身份与两段非学位经历均保留。；选定两篇论文及附勘误，不是完整书目；本人导师未披露，不能从合著者推断。必要摘录空格规范化和尾部国家/地点省略按原记录保留。</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K3"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -584,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -601,7 +655,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="60.2" customWidth="1" min="15" max="15"/>
+    <col width="65" customWidth="1" min="15" max="15"/>
     <col width="58.8" customWidth="1" min="16" max="16"/>
     <col width="65" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
@@ -1312,8 +1366,335 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2007-09</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2011-06</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>本人履历具体列Doctoral degree及南京大学Department of Mathematics &amp; IMS；2007-09至2011-06为原学习区间，不填授位日期。</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>吉林大学</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2002-09</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2004-07</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>本人履历具体列Master degree及吉林大学Institute of Mathematical Science；2002-09至2004-07为原学习区间，不填授位日期。</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Undergraduate degree（本科资格）</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>吉林大学</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>1998-09</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2002-07</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>本人履历具体列Undergraduate degree及吉林大学School of Mathematical Science，保留原本科资格英文称谓，不补专业；1998-09至2002-07不作授位日期。</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_training</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>北京大学北京国际数学研究中心</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2011-04</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2013-03</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2011-04至2013-03北京大学北京国际数学研究中心博士后，为非学位经历；与博士学习终2011-06重叠，保留原说不纠正时间。</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_training</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>新加坡国立大学</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2009-02-20</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>2009-04-05</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2009-02-20至2009-04-05新加坡国立大学数学系博士研究生访问，非独立授位，不提升为访学学位或导师。</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S10"/>
+  <autoFilter ref="A1:S15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -1324,6 +1705,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1545,7 +1931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1557,7 +1943,7 @@
     <col width="65" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
-    <col width="46.2" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
@@ -1680,12 +2066,102 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>$Q$-curvature flow on the standard sphere of even dimension</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文（来源书目）</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>官网原作者Xuezhang Chen、Xingwang Xu；J. Funct. Anal. 261，2011，934-980。仅官网书目，未核出版者或全文；不由合著者推本人导师。</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>The scalar curvature flow on $S^n$---perturbation theorem revisited</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文（来源书目）</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>官网原作者Xuezhang Chen、Xingwang Xu；Invent. Math. 187, no. 2，2012，395-506。原附勘误Invent. Math. 187(2012), no.2, 507–509，仅作品说明，不增第三篇。仅官网书目，未核出版者或全文；不由合著者推本人导师。</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:L4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1697,11 +2173,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="25.2" customWidth="1" min="2" max="2"/>
+    <col width="33.59999999999999" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -1968,8 +2444,41 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>陈学长</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>nju-chenxuezhang-profile</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://math.nju.edu.cn/szdw/apypl1/20190911/i21709.html</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G7"/>
+  <autoFilter ref="A1:G8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -1977,6 +2486,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>